<commit_message>
feat(F-NAR-019): ATOM-COL.POL.001-02 Le gâteau au citron de Chouchou
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-02.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-02.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le gâteau encore tiède de Chouchou</t>
+          <t>Le gâteau au citron de Chouchou</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine, palier, porte de la voisine</t>
+          <t>visite chez la voisine. Cuisine collante de zeste, fils jaunes, gâteau tiède, escalier à la cire, palier, thé à la menthe</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chouchou veut porter le gâteau au citron à la voisine. À la porte, il dit bonjour, s'il te plaît, merci.</t>
+          <t>Des fils jaunes collent au bois. Sur le gâteau, un éclat de zeste brille. Chouchou veut donner le plat maintenant. Elle saisit trop vite : l'éclat glisse. À la porte, elle avance trop vite : les mains n'attrapent pas, les mots se perdent. Elle refuse de foncer, attend, dit s'il te plaît. Merci vécu. Un bout trop vite : la cuillère glisse. Elle refuse, demande. Sur le bois, l'éclat de zeste tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le citron roule encore dans le saladier vide. Il fait un petit bruit de bois. Une tache jaune est sur le tablier de maman. Le gâteau refroidit près de la fenêtre ouverte. Une abeille passe dehors, sans entrer. Une goutte de glace sur la cuillère, tu vois ? Elle brille. On porte le plat à deux. Tes deux mains. Le torchon dessous. Il est doux. C'est pour la voisine. Oui. Elle a arrosé nos plantes. Les feuilles étaient toutes sèches. Maintenant elles sont vertes. Un peu, oui. On monte. L'escalier de l'immeuble sent la cire. Chaque marche fait un petit bruit de bois. On monte doucement. Tu tiens le plat. Il est lourd un peu. Je suis juste derrière. Le paillasson a une petite fleur brodée. En ce moment, Chouchou est devant la porte. Le plat reste au chaud entre ses mains. On sonne. Une fois. On entend des pas. Chouchou attend. Le plat tremble un tout petit peu. La porte s'ouvre. Une odeur de thé à la menthe sort. La voisine a un torchon à la main. Tu lui donnes, Chouchou. Chouchou avance le plat. Le citron sent encore, tout près.</t>
+          <t>Des fils jaunes collent au bois de la table. La table de la cuisine est collante de zeste. Chouchou connaît cette cuisine, un peu collante. Le gâteau au citron est tiède, tout rond. Une goutte de glace brille sur la cuillère. Elle brille, maman. On porte le plat à deux ? Oui, mes deux mains. Le torchon est dessous. Il est doux. Sur le gâteau, un éclat de zeste brille. Il est jaune, papa ! C'est le zeste, sur le dessus. Je le donne, maintenant ! Pendant que le plat est chaud ? Oui, tout de suite ! Chouchou saisit le plat trop vite. Le plat penche vers le bord. L'éclat de zeste glisse sur la glace. Oh. Tes deux mains, Chouchou ? Papa remet le plat droit. Oui, papa. Le torchon reste dessous ? Oui, maman. On monte ? On monte. L'escalier de l'immeuble sent la cire. Chaque marche fait un petit bruit de bois. Tu tiens le plat, Chouchou ? Il est lourd un peu. Je suis juste derrière toi. Le paillasson a une petite fleur brodée. En ce moment, Chouchou est devant la porte. On sonne, une fois ? Oui, une fois. La porte s'ouvre sur le palier. Une odeur de thé à la menthe sort. Bonjour. Bonjour. La voisine ouvre plus grand. C'est pour vous, maintenant ! Chouchou avance le plat trop vite. Le plat penche vers les mains ouvertes. Les mains ne le prennent pas. Oh. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu le donnes, Chouchou ? Papa s'accroupit à la même hauteur. Oui, papa. Les mots se perdent près de la porte. Personne n'entend la fin. Chouchou referme la bouche, un instant. Le plat reste lourd, tout chaud.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le citron roule encore dans le saladier vide. Il fait un petit bruit de bois. Une tache jaune est sur le tablier de maman. Le gâteau refroidit près de la fenêtre ouverte. Une abeille passe dehors, sans entrer. Une goutte de glace sur la cuillère, tu vois ? Elle brille. On porte le plat à deux. Tes deux mains. Le torchon dessous. Il est doux. C'est pour la voisine. Oui. Elle a arrosé nos plantes. Les feuilles étaient toutes sèches. Maintenant elles sont vertes. Un peu, oui. On monte. L'escalier de l'immeuble sent la cire. Chaque marche fait un petit bruit de bois. On monte doucement. Tu tiens le plat. Il est lourd un peu. Je suis juste derrière. Le paillasson a une petite fleur brodée. En ce moment, Chouchou est devant la porte. Le plat reste au chaud entre ses mains. On sonne. Une fois. On entend des pas. Chouchou attend. Le plat tremble un tout petit peu. La porte s'ouvre. Une odeur de thé à la menthe sort. La voisine a un torchon à la main. Tu lui donnes, Chouchou. Chouchou avance le plat. Le citron sent encore, tout près.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Des fils jaunes collent au bois de la table. La table de la cuisine est collante de zeste. Chouchou connaît cette cuisine, un peu collante. Le gâteau au citron est tiède, tout rond. Une goutte de glace brille sur la cuillère. Elle brille, maman. On porte le plat à deux ? Oui, mes deux mains. Le torchon est dessous. Il est doux. Sur le gâteau, un &lt;emphasis level="moderate"&gt;éclat de zeste&lt;/emphasis&gt; brille. Il est jaune, papa ! C'est le zeste, sur le dessus. Je le donne, maintenant ! Pendant que le plat est chaud ? Oui, tout de suite ! Chouchou saisit le plat trop vite. Le plat penche vers le bord. L'éclat de zeste glisse sur la glace. Oh. Tes deux mains, Chouchou ? Papa remet le plat droit. Oui, papa. Le torchon reste dessous ? Oui, maman. On monte ? On monte. L'escalier de l'immeuble sent la cire. Chaque marche fait un petit bruit de bois. Tu tiens le plat, Chouchou ? Il est lourd un peu. Je suis juste derrière toi. Le paillasson a une petite fleur brodée. En ce moment, Chouchou est devant la porte. On sonne, une fois ? Oui, une fois. La porte s'ouvre sur le palier. Une odeur de thé à la menthe sort. Bonjour. Bonjour. La voisine ouvre plus grand. C'est pour vous, maintenant ! Chouchou avance le plat trop vite. Le plat penche vers les mains ouvertes. Les mains ne le prennent pas. Oh. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu le donnes, Chouchou ? Papa s'accroupit à la même hauteur. Oui, papa. Les mots se perdent près de la porte. Personne n'entend la fin. Chouchou referme la bouche, un instant. Le plat reste lourd, tout chaud.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Zoé va chez la voisine avec papa. Papa sonne à la porte. La voisine ouvre. Zoé dit : &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Papa dit : bonjour. Ils apportent un gâteau au citron. Zoé tend le plat. Elle dit : s'il te plaît, c'est pour vous. La voisine sourit. Elle offre un verre d'eau. Zoé dit : merci. Papa dit : merci. Ils restent un moment. Zoé parle du parc. Au revoir, dit Zoé. La voisine dit : merci pour le gâteau. Papa serre la main de Zoé. Les mots sont là : bonjour, s'il te plaît, merci. [pause]</t>
+          <t>Des fils jaunes collent au bois de la table. La table de la cuisine est collante de zeste. Chouchou connaît cette cuisine, un peu collante. Le gâteau au citron est tiède, tout rond. Une goutte de glace brille sur la cuillère. Elle brille, maman. On porte le plat à deux ? Oui, mes deux mains. Le torchon est dessous. Il est doux. Sur le gâteau, un &lt;emphasis&gt;éclat de zeste&lt;/emphasis&gt; brille. Il est jaune, papa ! C'est le zeste, sur le dessus. Je le donne, maintenant ! Pendant que le plat est chaud ? Oui, tout de suite ! Chouchou saisit le plat trop vite. Le plat penche vers le bord. L'éclat de zeste glisse sur la glace. Oh. Tes deux mains, Chouchou ? Papa remet le plat droit. Oui, papa. Le torchon reste dessous ? Oui, maman. On monte ? On monte. L'escalier de l'immeuble sent la cire. Chaque marche fait un petit bruit de bois. Tu tiens le plat, Chouchou ? Il est lourd un peu. Je suis juste derrière toi. Le paillasson a une petite fleur brodée. En ce moment, Chouchou est devant la porte. On sonne, une fois ? Oui, une fois. La porte s'ouvre sur le palier. Une odeur de thé à la menthe sort. Bonjour. Bonjour. La voisine ouvre plus grand. C'est pour vous, maintenant ! Chouchou avance le plat trop vite. Le plat penche vers les mains ouvertes. Les mains ne le prennent pas. Oh. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu le donnes, Chouchou ? Papa s'accroupit à la même hauteur. Oui, papa. Les mots se perdent près de la porte. Personne n'entend la fin. Chouchou referme la bouche, un instant. Le plat reste lourd, tout chaud. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>éclat de zeste</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,47 +1326,68 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_donner_le_gateau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le citron roule encore dans le saladier vide.
-narrateur|Il fait un petit bruit de bois.
-narrateur|Une tache jaune est sur le tablier de maman.
-narrateur|Le gâteau refroidit près de la fenêtre ouverte.
-narrateur|Une abeille passe dehors, sans entrer.
-maman|Une goutte de glace sur la cuillère, tu vois ?
-enfant-m|Elle brille.
-papa|On porte le plat à deux.
-papa|Tes deux mains.
-maman|Le torchon dessous.
-maman|Il est doux.
-enfant-m|C'est pour la voisine.
-maman|Oui.
-maman|Elle a arrosé nos plantes.
-papa|Les feuilles étaient toutes sèches.
-enfant-m|Maintenant elles sont vertes.
-maman|Un peu, oui.
-papa|On monte.
+          <t>narrateur|Des fils jaunes collent au bois de la table.
+narrateur|La table de la cuisine est collante de zeste.
+narrateur|Chouchou connaît cette cuisine, un peu collante.
+narrateur|Le gâteau au citron est tiède, tout rond.
+maman|Une goutte de glace brille sur la cuillère.
+enfant-f|Elle brille, maman.
+papa|On porte le plat à deux ?
+enfant-f|Oui, mes deux mains.
+maman|Le torchon est dessous.
+enfant-f|Il est doux.
+narrateur|Sur le gâteau, un éclat de zeste brille.
+enfant-f|Il est jaune, papa !
+papa|C'est le zeste, sur le dessus.
+enfant-f|Je le donne, maintenant !
+maman|Pendant que le plat est chaud ?
+enfant-f|Oui, tout de suite !
+narrateur|Chouchou saisit le plat trop vite.
+narrateur|Le plat penche vers le bord.
+narrateur|L'éclat de zeste glisse sur la glace.
+enfant-f|Oh.
+papa|Tes deux mains, Chouchou ?
+narrateur|Papa remet le plat droit.
+enfant-f|Oui, papa.
+maman|Le torchon reste dessous ?
+enfant-f|Oui, maman.
+papa|On monte ?
+enfant-f|On monte.
 narrateur|L'escalier de l'immeuble sent la cire.
 narrateur|Chaque marche fait un petit bruit de bois.
-papa|On monte doucement.
-papa|Tu tiens le plat.
-enfant-m|Il est lourd un peu.
-maman|Je suis juste derrière.
+papa|Tu tiens le plat, Chouchou ?
+enfant-f|Il est lourd un peu.
+maman|Je suis juste derrière toi.
 narrateur|Le paillasson a une petite fleur brodée.
 narrateur|En ce moment, Chouchou est devant la porte.
-narrateur|Le plat reste au chaud entre ses mains.
-papa|On sonne.
-papa|Une fois.
-narrateur|On entend des pas.
-narrateur|Chouchou attend.
-narrateur|Le plat tremble un tout petit peu.
-narrateur|La porte s'ouvre.
+papa|On sonne, une fois ?
+enfant-f|Oui, une fois.
+narrateur|La porte s'ouvre sur le palier.
 narrateur|Une odeur de thé à la menthe sort.
-narrateur|La voisine a un torchon à la main.
-maman|Tu lui donnes, Chouchou.
-narrateur|Chouchou avance le plat.
-narrateur|Le citron sent encore, tout près.</t>
+enfant-f|Bonjour.
+papa|Bonjour.
+narrateur|La voisine ouvre plus grand.
+enfant-f|C'est pour vous, maintenant !
+narrateur|Chouchou avance le plat trop vite.
+narrateur|Le plat penche vers les mains ouvertes.
+narrateur|Les mains ne le prennent pas.
+enfant-f|Oh.
+narrateur|Le sourire de Chouchou disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+papa|Tu le donnes, Chouchou ?
+narrateur|Papa s'accroupit à la même hauteur.
+enfant-f|Oui, papa.
+narrateur|Les mots se perdent près de la porte.
+narrateur|Personne n'entend la fin.
+narrateur|Chouchou referme la bouche, un instant.
+narrateur|Le plat reste lourd, tout chaud.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1398,17 +1419,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou donne le gâteau. Que dit-il ?</t>
+          <t>Chouchou donne le gâteau. Que dit-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou donne le gâteau. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Chouchou donne le &lt;emphasis level="moderate"&gt;gâteau&lt;/emphasis&gt;. Que dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Zoé donne le gâteau. Que dit-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Chouchou donne le &lt;emphasis&gt;gâteau&lt;/emphasis&gt;. Que dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1433,7 +1454,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il dit s'il te plaît et merci. Que dit Chouchou ?</t>
+          <t>Elle dit s'il te plaît et merci. Que dit Chouchou ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1471,7 +1492,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1482,7 +1503,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1497,34 +1518,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>gâteau</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1539,23 +1564,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_dit_s_il_te_plait_en_tendant_le_plat; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
           <t>narrateur|Chouchou donne le gâteau.
-narrateur|Que dit-il ?</t>
+narrateur|Que dit-elle ?</t>
         </is>
       </c>
     </row>
@@ -1582,17 +1607,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. S'il te plaît. C'est pour vous. C'est un gâteau au citron. Le plat passe de Chouchou à ses mains. Il n'est plus lourd. Un verre d'eau arrive, tout clair. Merci. Merci. Merci pour l'eau. Ils restent un moment sur le palier clair. Tu parles du parc, si tu veux. Les balançoires sont vertes. On dit au revoir, maintenant. Au revoir. Une lumière jaune vient de la porte ouverte. L'odeur de citron reste dans l'escalier. Elle l'a pris. Oui. Elle l'a pris.</t>
+          <t>Chouchou avance le plat trop vite. Le gâteau, le citron, pour vous ! Les mots se bousculent dans sa bouche. Les mains ouvertes n'attrapent pas le plat. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle recule le plat, un peu. Le plat est chaud, Chouchou ? Papa reste à sa hauteur. La fleur du paillasson est sous tes pieds. Maman n'a pas fini non plus. Chouchou attend que le silence arrive. Sur le dessus, l'éclat de zeste brille. Il est là. S'il te plaît. C'est pour vous. Le plat passe dans des mains calmes. Le plat n'est plus lourd. Merci, Chouchou. Papa a entendu toute la phrase. Un verre d'eau arrive, tout clair. Merci. Tu as soif, un peu ? Un peu, maman. Tu parles du parc, si tu veux ? Les balançoires sont vertes. On rentre, Chouchou ? Au revoir. Une lumière jaune vient de la porte ouverte. L'odeur de citron reste dans l'escalier.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. S'il te plaît. C'est pour vous. C'est un gâteau au citron. Le plat passe de Chouchou à ses mains. Il n'est plus lourd. Un verre d'eau arrive, tout clair. Merci. Merci. Merci pour l'eau. Ils restent un moment sur le palier clair. Tu parles du parc, si tu veux. Les balançoires sont vertes. On dit au revoir, maintenant. Au revoir. Une lumière jaune vient de la porte ouverte. L'odeur de citron reste dans l'escalier. Elle l'a pris. Oui. Elle l'a pris.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou avance le plat trop vite. Le gâteau, le citron, pour vous ! Les mots se bousculent dans sa bouche. Les mains ouvertes n'attrapent pas le plat. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle recule le plat, un peu. Le plat est chaud, Chouchou ? Papa reste à sa hauteur. La fleur du paillasson est sous tes pieds. Maman n'a pas fini non plus. Chouchou attend que le silence arrive. Sur le dessus, l'éclat de zeste brille. Il est là. &lt;emphasis level="moderate"&gt;S'il te plaît&lt;/emphasis&gt;. C'est pour vous. Le plat passe dans des mains calmes. Le plat n'est plus lourd. Merci, Chouchou. Papa a entendu toute la phrase. Un verre d'eau arrive, tout clair. Merci. Tu as soif, un peu ? Un peu, maman. Tu parles du parc, si tu veux ? Les balançoires sont vertes. On rentre, Chouchou ? Au revoir. Une lumière jaune vient de la porte ouverte. L'odeur de citron reste dans l'escalier.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Zoé a dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Elle a dit s'il te plaît. Elle a dit merci. Papa était avec elle. [pause]</t>
+          <t>Chouchou avance le plat trop vite. Le gâteau, le citron, pour vous ! Les mots se bousculent dans sa bouche. Les mains ouvertes n'attrapent pas le plat. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle recule le plat, un peu. Le plat est chaud, Chouchou ? Papa reste à sa hauteur. La fleur du paillasson est sous tes pieds. Maman n'a pas fini non plus. Chouchou attend que le silence arrive. Sur le dessus, l'éclat de zeste brille. Il est là. &lt;emphasis&gt;S'il te plaît&lt;/emphasis&gt;. C'est pour vous. Le plat passe dans des mains calmes. Le plat n'est plus lourd. Merci, Chouchou. Papa a entendu toute la phrase. Un verre d'eau arrive, tout clair. Merci. Tu as soif, un peu ? Un peu, maman. Tu parles du parc, si tu veux ? Les balançoires sont vertes. On rentre, Chouchou ? Au revoir. Une lumière jaune vient de la porte ouverte. L'odeur de citron reste dans l'escalier. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1639,7 +1664,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1647,10 +1672,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1673,30 +1698,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>S'il te plaît</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1705,10 +1730,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1721,32 +1746,47 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_puis_tend_le_plat; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|Bonjour.
-papa|Bonjour.
-enfant-m|S'il te plaît.
-enfant-m|C'est pour vous.
-papa|C'est un gâteau au citron.
-narrateur|Le plat passe de Chouchou à ses mains.
-narrateur|Il n'est plus lourd.
+          <t>narrateur|Chouchou avance le plat trop vite.
+enfant-f|Le gâteau, le citron, pour vous !
+narrateur|Les mots se bousculent dans sa bouche.
+narrateur|Les mains ouvertes n'attrapent pas le plat.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Chouchou refuse de foncer.
+narrateur|Elle recule le plat, un peu.
+papa|Le plat est chaud, Chouchou ?
+narrateur|Papa reste à sa hauteur.
+maman|La fleur du paillasson est sous tes pieds.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Chouchou attend que le silence arrive.
+narrateur|Sur le dessus, l'éclat de zeste brille.
+enfant-f|Il est là.
+enfant-f|S'il te plaît.
+enfant-f|C'est pour vous.
+narrateur|Le plat passe dans des mains calmes.
+narrateur|Le plat n'est plus lourd.
+papa|Merci, Chouchou.
+narrateur|Papa a entendu toute la phrase.
 narrateur|Un verre d'eau arrive, tout clair.
-enfant-m|Merci.
-maman|Merci.
-papa|Merci pour l'eau.
-narrateur|Ils restent un moment sur le palier clair.
-papa|Tu parles du parc, si tu veux.
-enfant-m|Les balançoires sont vertes.
-maman|On dit au revoir, maintenant.
-enfant-m|Au revoir.
+enfant-f|Merci.
+maman|Tu as soif, un peu ?
+enfant-f|Un peu, maman.
+papa|Tu parles du parc, si tu veux ?
+enfant-f|Les balançoires sont vertes.
+maman|On rentre, Chouchou ?
+enfant-f|Au revoir.
 narrateur|Une lumière jaune vient de la porte ouverte.
-narrateur|L'odeur de citron reste dans l'escalier.
-enfant-m|Elle l'a pris.
-papa|Oui.
-papa|Elle l'a pris.</t>
+narrateur|L'odeur de citron reste dans l'escalier.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>porte,verre</t>
         </is>
       </c>
     </row>
@@ -1773,17 +1813,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Chouchou redescend l'escalier avec papa et maman. Le bois ciré sent encore un peu. Le citron reste dans l'air. Tu as porté le plat. Tes deux mains. Il n'est plus lourd. Non. Il est chez elle. Une miette jaune reste sur le torchon. On la met dans l'évier. À la maison, le citron est encore dans le saladier. La cuillère brille près de la fenêtre. L'abeille n'est plus là. Le gâteau non plus. Il est monté. Oui. Je l'ai donné. Les plantes ont de l'eau, maintenant. Et elle a du gâteau. Il était encore tiède. Oui. Tout rond.</t>
+          <t>Chouchou redescend l'escalier avec papa et maman. Le bois ciré sent la cire, un peu. Le citron reste dans l'air. Le plat n'est plus lourd, papa. Elle l'a pris, oui. À la maison, la table a des zestes. La cuillère brille près du bois collant. Je prends un bout, maintenant ! Chouchou avance la main trop vite. La cuillère glisse vers le bord. Oh. Papa n'a pas fini sa phrase. La table est collante, Chouchou. Les deux voix se mélangent. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute la cuisine, un instant. Elle pose la main, sans presser. S'il te plaît, un bout ? Oui, un petit. Il est tiède, maman. Tu restes un peu ? Oui, papa. Le torchon est près de l'évier. On le met ? Oui, dans l'eau. Le bout de gâteau sent le citron. Il colle aux doigts. Comme la table, oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Chouchou redescend l'escalier avec papa et maman. Le bois ciré sent encore un peu. Le citron reste dans l'air. Tu as porté le plat. Tes deux mains. Il n'est plus lourd. Non. Il est chez elle. Une miette jaune reste sur le torchon. On la met dans l'évier. À la maison, le citron est encore dans le saladier. La cuillère brille près de la fenêtre. L'abeille n'est plus là. Le gâteau non plus. Il est monté. Oui. Je l'ai donné. Les plantes ont de l'eau, maintenant. Et elle a du gâteau. Il était encore tiède. Oui. Tout rond.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou redescend l'escalier avec papa et maman. Le bois ciré sent la cire, un peu. Le citron reste dans l'air. Le plat n'est plus lourd, papa. Elle l'a pris, oui. À la maison, la table a des zestes. La &lt;emphasis level="moderate"&gt;cuillère&lt;/emphasis&gt; brille près du bois collant. Je prends un bout, maintenant ! Chouchou avance la main trop vite. La cuillère glisse vers le bord. Oh. Papa n'a pas fini sa phrase. La table est collante, Chouchou. Les deux voix se mélangent. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute la cuisine, un instant. Elle pose la main, sans presser. S'il te plaît, un bout ? Oui, un petit. Il est tiède, maman. Tu restes un peu ? Oui, papa. Le torchon est près de l'évier. On le met ? Oui, dans l'eau. Le bout de gâteau sent le citron. Il colle aux doigts. Comme la table, oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Zoé redescend l'escalier avec papa. Le citron sent encore. [pause]</t>
+          <t>Chouchou redescend l'escalier avec papa et maman. Le bois ciré sent la cire, un peu. Le citron reste dans l'air. Le plat n'est plus lourd, papa. Elle l'a pris, oui. À la maison, la table a des zestes. La &lt;emphasis&gt;cuillère&lt;/emphasis&gt; brille près du bois collant. Je prends un bout, maintenant ! Chouchou avance la main trop vite. La cuillère glisse vers le bord. Oh. Papa n'a pas fini sa phrase. La table est collante, Chouchou. Les deux voix se mélangent. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute la cuisine, un instant. Elle pose la main, sans presser. S'il te plaît, un bout ? Oui, un petit. Il est tiède, maman. Tu restes un peu ? Oui, papa. Le torchon est près de l'évier. On le met ? Oui, dans l'eau. Le bout de gâteau sent le citron. Il colle aux doigts. Comme la table, oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1830,7 +1870,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1838,10 +1878,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1862,28 +1902,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>cuillère</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1892,10 +1936,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1906,36 +1950,48 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sur_la_cuillere; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
           <t>narrateur|Chouchou redescend l'escalier avec papa et maman.
-narrateur|Le bois ciré sent encore un peu.
+narrateur|Le bois ciré sent la cire, un peu.
 narrateur|Le citron reste dans l'air.
-maman|Tu as porté le plat.
-papa|Tes deux mains.
-enfant-m|Il n'est plus lourd.
-maman|Non.
-maman|Il est chez elle.
-narrateur|Une miette jaune reste sur le torchon.
-maman|On la met dans l'évier.
-narrateur|À la maison, le citron est encore dans le saladier.
-narrateur|La cuillère brille près de la fenêtre.
-papa|L'abeille n'est plus là.
-enfant-m|Le gâteau non plus.
-maman|Il est monté.
-enfant-m|Oui.
-enfant-m|Je l'ai donné.
-papa|Les plantes ont de l'eau, maintenant.
-maman|Et elle a du gâteau.
-enfant-m|Il était encore tiède.
-papa|Oui.
-papa|Tout rond.</t>
+enfant-f|Le plat n'est plus lourd, papa.
+papa|Elle l'a pris, oui.
+narrateur|À la maison, la table a des zestes.
+narrateur|La cuillère brille près du bois collant.
+enfant-f|Je prends un bout, maintenant !
+narrateur|Chouchou avance la main trop vite.
+narrateur|La cuillère glisse vers le bord.
+enfant-f|Oh.
+narrateur|Papa n'a pas fini sa phrase.
+papa|La table est collante, Chouchou.
+narrateur|Les deux voix se mélangent.
+enfant-f|Oh.
+narrateur|Chouchou refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Elle écoute la cuisine, un instant.
+narrateur|Elle pose la main, sans presser.
+enfant-f|S'il te plaît, un bout ?
+maman|Oui, un petit.
+enfant-f|Il est tiède, maman.
+papa|Tu restes un peu ?
+enfant-f|Oui, papa.
+maman|Le torchon est près de l'évier.
+enfant-f|On le met ?
+papa|Oui, dans l'eau.
+narrateur|Le bout de gâteau sent le citron.
+enfant-f|Il colle aux doigts.
+maman|Comme la table, oui.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>pas,table</t>
         </is>
       </c>
     </row>
@@ -1962,17 +2018,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le citron sent encore, tout bas. Le saladier est vide, à part lui. Bonne soirée, Chouchou. Le plat n'est plus lourd.</t>
+          <t>Ils restent près de la table collante. Les fils jaunes tiennent sur le bois. Comme sur le gâteau, papa. Tu le vois, toi ? Oui, sur le bois. On est bien, ici. Chouchou glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Le plat est rentré vide. Oui, elle l'a pris. L'odeur de citron reste dans la cuisine. Il est là, maman. Oui, sur le bois. L'éclat de zeste tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le citron sent encore, tout bas. Le saladier est vide, à part lui. Bonne soirée, Chouchou. Le plat n'est plus lourd.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table collante. Les fils jaunes tiennent sur le bois. Comme sur le gâteau, papa. Tu le vois, toi ? Oui, sur le bois. On est bien, ici. Chouchou glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Le plat est rentré vide. Oui, elle l'a pris. L'odeur de citron reste dans la cuisine. Il est là, maman. Oui, sur le bois. L'&lt;emphasis level="moderate"&gt;éclat de zeste&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table collante. Les fils jaunes tiennent sur le bois. Comme sur le gâteau, papa. Tu le vois, toi ? Oui, sur le bois. On est bien, ici. Chouchou glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Le plat est rentré vide. Oui, elle l'a pris. L'odeur de citron reste dans la cuisine. Il est là, maman. Oui, sur le bois. L'&lt;emphasis&gt;éclat de zeste&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2019,7 +2075,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2027,10 +2083,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2039,12 +2095,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2053,17 +2109,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de zeste</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2072,11 +2132,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2085,27 +2145,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le citron sent encore, tout bas.
-narrateur|Le saladier est vide, à part lui.
-maman|Bonne soirée, Chouchou.
-papa|Le plat n'est plus lourd.</t>
+          <t>narrateur|Ils restent près de la table collante.
+narrateur|Les fils jaunes tiennent sur le bois.
+enfant-f|Comme sur le gâteau, papa.
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur le bois.
+maman|On est bien, ici.
+narrateur|Chouchou glisse le doigt, sans se presser.
+enfant-f|On le sent, maman.
+maman|Tu le sens sur tes doigts ?
+enfant-f|Oui, il colle.
+papa|Le plat est rentré vide.
+enfant-f|Oui, elle l'a pris.
+narrateur|L'odeur de citron reste dans la cuisine.
+enfant-f|Il est là, maman.
+maman|Oui, sur le bois.
+narrateur|L'éclat de zeste tient sur le bois.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>table,cuisine</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2211,6 +2292,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>